<commit_message>
Material row insertion, report improvements, and UI enhancements
- Fix materials silently dropped when block K column is full — now inserts row before 总开销
- Worker/site totals exclude unmatched entries; split gas from ticket as separate columns
- Add input validation warnings for missing address or worker fields
- Add Labor and Subtotal columns to Extracted Worker Data table with per-worker subtotals
- Remove Rate column from Employee Totals
- Remove dead droppedMaterials field from ProcessResult
- Expand smoke test to 53 checks covering material insertion, warnings, and totals

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-input.xlsx
+++ b/test-input.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
   <si>
     <t>Name</t>
   </si>
@@ -68,6 +68,9 @@
   </si>
   <si>
     <t>6033</t>
+  </si>
+  <si>
+    <t>4444</t>
   </si>
 </sst>
 </file>
@@ -444,7 +447,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:I15"/>
+  <dimension ref="B1:I17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="2:9" x14ac:dyDescent="0.25">
@@ -509,115 +512,128 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D5" t="s">
+    <row r="5" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D6" t="s">
+    <row r="7" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
         <v>11</v>
       </c>
-      <c r="E6">
+      <c r="E7">
         <v>10</v>
       </c>
-      <c r="G6">
+      <c r="G7">
         <v>300</v>
       </c>
     </row>
-    <row r="7" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D7" t="s">
+    <row r="8" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
         <v>12</v>
       </c>
-      <c r="E7">
+      <c r="E8">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
         <v>14</v>
       </c>
-      <c r="C9">
+      <c r="C10">
         <v>13</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D10" t="s">
         <v>8</v>
       </c>
-      <c r="H9">
+      <c r="H10">
         <v>25</v>
       </c>
-      <c r="I9">
+      <c r="I10">
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D10" t="s">
+    <row r="11" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D11" t="s">
         <v>15</v>
       </c>
-      <c r="E10">
+      <c r="E11">
         <v>12</v>
       </c>
-      <c r="G10">
+      <c r="G11">
         <v>500</v>
       </c>
     </row>
-    <row r="11" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D11" t="s">
+    <row r="12" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D12" t="s">
         <v>16</v>
       </c>
-      <c r="E11">
+      <c r="E12">
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D12" t="s">
+    <row r="13" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D13" t="s">
         <v>9</v>
       </c>
-      <c r="E12">
+      <c r="E13">
         <v>15</v>
       </c>
-      <c r="G12">
+      <c r="G13">
         <v>800</v>
       </c>
-      <c r="H12">
+      <c r="H13">
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
         <v>17</v>
       </c>
-      <c r="C14">
+      <c r="C15">
         <v>18</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D15" t="s">
         <v>18</v>
       </c>
-      <c r="E14">
+      <c r="E15">
         <v>24</v>
       </c>
-      <c r="G14">
+      <c r="G15">
         <v>1200</v>
       </c>
-      <c r="H14">
+      <c r="H15">
         <v>50</v>
       </c>
-      <c r="I14">
+      <c r="I15">
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B15" t="s">
+    <row r="16" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D16" t="s">
+        <v>19</v>
+      </c>
+      <c r="G16">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>